<commit_message>
Add recurring reference workflow and capacity safeguards
</commit_message>
<xml_diff>
--- a/s04_web_visualization/public/data/data_dictionary.xlsx
+++ b/s04_web_visualization/public/data/data_dictionary.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="READ ME" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="READ ME" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Columns" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Enums" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -497,7 +497,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dataset: Chinese overseas renewable-energy &amp; related projects. Data as of 2026-07-30. 3527 rows covering 1987 projects (incl. 312 transmission and 136 manufacturing projects).</t>
+          <t>Dataset scope: Chinese overseas renewable-energy and related projects. This workbook defines the CSV grain, fields, applicability, units and controlled values.</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>2. CAPACITY SEMANTICS — three different 'capacities', two different units</t>
+          <t>2. CAPACITY &amp; ENERGY-MIX SEMANTICS — keep generation, storage and manufacturing metrics separate</t>
         </is>
       </c>
     </row>
@@ -580,94 +580,81 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>• Integrated Energy (hybrid, e.g. solar+storage plants): capacity_mw is the plant total; pv_capacity_mw is the PV sub-component; storage_* are the storage sub-component. Sub-components need not sum to the total.</t>
+          <t>• Integrated Energy means a mixed generation system (renewable and/or thermal sources). capacity_mw is total generation capacity; pv_capacity_mw is a separately captured PV component when available; storage_* are separate storage metrics. Do not infer missing component capacities from names or totals.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>• storage_* fields appear on ANY project that disclosed them (mostly Energy Storage and Integrated Energy · Solar + Storage) — filter by field presence, not only by category.</t>
+          <t>• generation_sources stores pipe-separated atomic generation-source keys; storage is never a generation source. storage_status records evidence strength, while technology_tags_cn/_en provides controlled combination labels such as Solar + Storage, Wind + Storage or Wind + Solar + Storage.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr"/>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>• storage_* fields may appear on Solar PV, Wind Power, Integrated Energy or Energy Storage projects. Filter by field presence or storage_status/technology tags, not only by category.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>3. COLUMN APPLICABILITY BY CATEGORY — which columns mean anything for which projects</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>Column group</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Generation (PV/Wind/Hydro/Geo/Biomass)</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>Energy Storage</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>Integrated Energy (hybrid)</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>Transmission</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>Manufacturing</t>
         </is>
       </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>capacity_mw</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="inlineStr"/>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>✓ (plant total)</t>
-        </is>
-      </c>
-      <c r="E20" s="7" t="inlineStr"/>
-      <c r="F20" s="7" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>subcategory_cn / _en</t>
+          <t>capacity_mw</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>✓ Solar PV only (Utility-scale/Distributed)</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr"/>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>✓ (Solar + Storage / Other)</t>
+          <t>✓ (plant total)</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr"/>
@@ -676,38 +663,34 @@
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>pv_capacity_mw</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr"/>
+          <t>subcategory_cn / _en</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>✓ Solar PV only (Utility-scale/Distributed)</t>
+        </is>
+      </c>
       <c r="C22" s="7" t="inlineStr"/>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>✓ (PV sub-component)</t>
-        </is>
-      </c>
+      <c r="D22" s="7" t="inlineStr"/>
       <c r="E22" s="7" t="inlineStr"/>
       <c r="F22" s="7" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>storage_power_mw / storage_energy_mwh</t>
+          <t>generation_sources</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>if disclosed</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+          <t>✓ atomic generation source(s)</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr"/>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>✓ (storage sub-component)</t>
+          <t>✓ mixed generation source(s)</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr"/>
@@ -716,128 +699,196 @@
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>voltage_kv / line_length_km / transmission_capacity_mw</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="inlineStr"/>
-      <c r="C24" s="7" t="inlineStr"/>
-      <c r="D24" s="7" t="inlineStr"/>
-      <c r="E24" s="7" t="inlineStr">
+          <t>storage_status / technology_tags_*</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>if storage/combination disclosed</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>if storage/combination disclosed</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr"/>
       <c r="F24" s="7" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>production_capacity_value / _unit</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr"/>
+          <t>pv_capacity_mw</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>if separately captured</t>
+        </is>
+      </c>
       <c r="C25" s="7" t="inlineStr"/>
-      <c r="D25" s="7" t="inlineStr"/>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>if separately captured</t>
+        </is>
+      </c>
       <c r="E25" s="7" t="inlineStr"/>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="F25" s="7" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
+          <t>storage_power_mw / storage_energy_mwh</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>if disclosed</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>✓ (storage sub-component)</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr"/>
+      <c r="F26" s="7" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>voltage_kv / line_length_km / transmission_capacity_mw</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr"/>
+      <c r="C27" s="7" t="inlineStr"/>
+      <c r="D27" s="7" t="inlineStr"/>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>production_capacity_value / _unit</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr"/>
+      <c r="C28" s="7" t="inlineStr"/>
+      <c r="D28" s="7" t="inlineStr"/>
+      <c r="E28" s="7" t="inlineStr"/>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
           <t>stage / year / month / entities / amounts</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E26" s="7" t="inlineStr">
+      <c r="E29" s="7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F26" s="7" t="inlineStr">
+      <c r="F29" s="7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>• Blank cells above = the column is not applicable to that category (structurally empty, not missing data).</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>• Manufacturing capacities use HETEROGENEOUS units (GW/year, GWh/year, t/year). Values originally in 10,000 tonnes/year are multiplied by 10,000 for t/year. Never sum production_capacity_value across different units.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>4. GENERAL CONVENTIONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>• Blank = not disclosed in sources, NOT zero.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>• All monetary fields are in MILLION USD. contract_amount_usd / financing_amount_usd are only collected for events from July 2026 onward; earlier events are blank by policy (not missing).</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>• is_central_soe describes the Chinese ENTITY on that row (1/0), not the project; a project may mix SOE and non-SOE rows.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>• Scope baseline: milestone events from 2022 onward; projects whose latest event predates 2022 are excluded; projects located in mainland China / Hong Kong / Macau / Taiwan are excluded.</t>
+          <t>• Blank = not disclosed in sources, NOT zero.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>• Row order is for human browsing only (generation+storage block, then transmission, then manufacturing; sorted by canonical_id, event_id inside each block). Do not rely on row order programmatically.</t>
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>• All monetary fields are in MILLION USD. contract_amount_usd / financing_amount_usd are only collected for events from July 2026 onward; earlier events are blank by policy (not missing).</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>• is_central_soe describes the Chinese ENTITY on that row (1/0), not the project; a project may mix SOE and non-SOE rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>• Scope baseline: milestone events from 2022 onward; projects whose latest event predates 2022 are excluded; projects located in mainland China / Hong Kong / Macau / Taiwan are excluded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>• Row order is for human browsing only (generation+storage block, then transmission, then manufacturing; sorted by canonical_id, event_id inside each block). Do not rely on row order programmatically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>• Stage vocabulary: fine-grained stage_cn/_en roll up to four macro groups (stage_group_*): Pre-construction / In Construction / Construction Completed / Acquired — see the Enums sheet.</t>
         </is>
@@ -1091,12 +1142,12 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Project subcategory in Chinese. Solar PV: 集中式 (utility-scale; default when unspecified) / 分布式 (distributed). Integrated Energy: 光储 (solar+storage) / 其他 (other; default). Blank for other categories.</t>
+          <t>Project-form subcategory in Chinese. Solar PV only: 集中式 (utility-scale; default when unspecified) / 分布式 (distributed). Energy combinations are stored in technology_tags_cn/_en, not subcategory.</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Solar PV, Integrated Energy</t>
+          <t>Solar PV only</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -1113,12 +1164,12 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Project subcategory in English (Utility-scale / Distributed / Solar + Storage / Other).</t>
+          <t>Project-form subcategory in English (Utility-scale / Distributed). Energy combinations are stored in technology_tags_cn/_en.</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Solar PV, Integrated Energy</t>
+          <t>Solar PV only</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -1135,7 +1186,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Generation sources in Chinese, separated by ' | '. Event-level source facts; blank when not disclosed.</t>
+          <t>Event-level pipe-separated atomic generation-source keys in Chinese (e.g. 光伏 | 风电). Energy storage is excluded by definition; blank means no structured source fact was determined.</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
@@ -1157,12 +1208,12 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Storage evidence status: confirmed / planned / optional / unclear / not_mentioned. Storage power and energy are exported only when confirmed.</t>
+          <t>Controlled storage-evidence status: confirmed / planned / optional / unclear / not_mentioned. Only confirmed storage exports numeric storage_* values.</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Generation, Integrated Energy &amp; Energy Storage</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -1179,17 +1230,17 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Project-level technology tags in Chinese, separated by ' | '. Repeated for all events and entities of the project.</t>
+          <t>Pipe-separated controlled Chinese technology-combination labels (光储 / 风储 / 风光 / 风光储). These project-level labels repeat for every event and entity and are independent of project-form subcategory.</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Generation &amp; Integrated Energy</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>光储</t>
+          <t>风光储</t>
         </is>
       </c>
     </row>
@@ -1201,17 +1252,17 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>English equivalents of technology_tags_cn, separated by ' | '.</t>
+          <t>English rendering of technology_tags_cn (Solar + Storage / Wind + Storage / Wind + Solar / Wind + Solar + Storage).</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Generation &amp; Integrated Energy</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Solar + Storage</t>
+          <t>Wind + Solar + Storage</t>
         </is>
       </c>
     </row>
@@ -1377,12 +1428,12 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Solar PV sub-component capacity in MW, for Integrated Energy (hybrid) projects only.</t>
+          <t>Separately captured Solar PV component capacity in MW, when disclosed. Most common in solar+storage and Integrated Energy projects; blank otherwise.</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Integrated Energy</t>
+          <t>Any project with a separately captured PV component</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -1842,7 +1893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:E37"/>
+  <dimension ref="A2:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2067,7 +2118,7 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>capacity_mw (MW), optional pv/storage sub-metrics</t>
+          <t>total generation capacity_mw (MW), plus disclosed pv/storage sub-metrics</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -2392,7 +2443,7 @@
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>Subcategories (Solar PV &amp; Integrated Energy only)</t>
+          <t>Project-form subcategories (Solar PV only)</t>
         </is>
       </c>
     </row>
@@ -2461,65 +2512,415 @@
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>Manufacturing production-capacity units (never sum across units)</t>
+          <t>Atomic generation sources (energy storage is excluded)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Key (zh)</t>
         </is>
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>Meaning</t>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>Order</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>GW/year</t>
+          <t>光伏</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>GW per year (module/cell manufacturing lines)</t>
-        </is>
+          <t>Solar PV</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>GWh/year</t>
+          <t>风电</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>GWh per year (battery factories)</t>
-        </is>
+          <t>Wind Power</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>t/year</t>
+          <t>水电</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Tonnes per year (polysilicon/materials); source 10k-tonne values multiplied by 10,000</t>
-        </is>
+          <t>Hydropower</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
+          <t>地热及余热</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Geothermal &amp; Waste Heat</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>生物质</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Biomass</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>核电</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Nuclear Power</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>火电</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Thermal Power</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>Storage evidence status</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>confirmed</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>已确认配储</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>拟配储</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>可选配储</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>含糊</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>not_mentioned</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>未提及</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>Not Mentioned</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>Technology combination tags (independent of subcategory)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="10" t="inlineStr">
+        <is>
+          <t>Key (zh)</t>
+        </is>
+      </c>
+      <c r="B51" s="10" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="C51" s="10" t="inlineStr">
+        <is>
+          <t>Allowed project categories</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>光储</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Solar + Storage</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>光伏</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>风储</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Wind + Storage</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>风电</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>风光</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Wind + Solar</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>综合能源</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="inlineStr">
+        <is>
+          <t>风光储</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>Wind + Solar + Storage</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>综合能源</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="9" t="inlineStr">
+        <is>
+          <t>Manufacturing production-capacity units (never sum across units)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="B58" s="10" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="7" t="inlineStr">
+        <is>
+          <t>GW/year</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>GW per year (module/cell manufacturing lines)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="7" t="inlineStr">
+        <is>
+          <t>GWh/year</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>GWh per year (battery factories)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="7" t="inlineStr">
+        <is>
+          <t>t/year</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>Tonnes per year (polysilicon/materials); source 10k-tonne values multiplied by 10,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="B37" s="7" t="inlineStr">
+      <c r="B62" s="7" t="inlineStr">
         <is>
           <t>value disclosed without a usable unit</t>
         </is>

</xml_diff>